<commit_message>
fix: honor custom width and height on barcode and qr code in html and pdf outputs
</commit_message>
<xml_diff>
--- a/templates/INVOICE_REPORT.xlsx
+++ b/templates/INVOICE_REPORT.xlsx
@@ -1,75 +1,156 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\ApexReports\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10305"/>
   </bookViews>
   <sheets>
-    <sheet name="Invoice" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Invoice" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Invoice'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$6:$6</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+  <si>
+    <t>TAX INVOICE</t>
+  </si>
+  <si>
+    <t>{{company.name}}</t>
+  </si>
+  <si>
+    <t>Invoice No: {{invoice_no}}</t>
+  </si>
+  <si>
+    <t>Bill To: {{customer.name}}</t>
+  </si>
+  <si>
+    <t>Date: {{invoice_date}}</t>
+  </si>
+  <si>
+    <t>Item Code</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Unit Price</t>
+  </si>
+  <si>
+    <t>Line Total</t>
+  </si>
+  <si>
+    <t>{{#each items}}</t>
+  </si>
+  <si>
+    <t>{{item_code}}</t>
+  </si>
+  <si>
+    <t>{{description}}</t>
+  </si>
+  <si>
+    <t>{{qty}}</t>
+  </si>
+  <si>
+    <t>{{unit_price}}</t>
+  </si>
+  <si>
+    <t>{{/each}}</t>
+  </si>
+  <si>
+    <t>Subtotal:</t>
+  </si>
+  <si>
+    <t>Scan to verify:</t>
+  </si>
+  <si>
+    <t>{{#each invoices page_break=true}}</t>
+  </si>
+  <si>
+    <t>{{@barcode invoice_no format=code128 width=40 height=5}}</t>
+  </si>
+  <si>
+    <t>{{@qr 'https://verify.apex.corp/inv/' + invoice_no width=30 height=30}}</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF1E3A8A"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001E3A8A"/>
-      <sz val="18"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1E293B"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001E293B"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF334155"/>
       <name val="Calibri"/>
-      <color rgb="00334155"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
+        <fgColor rgb="FF1E3A8A"/>
+        <bgColor rgb="FF1E3A8A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,119 +164,64 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </right>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="12">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -483,149 +509,119 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>TAX INVOICE</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>{{@barcode invoice_no format=code128 width=140 height=35}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>{{company.name}}</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Invoice No: {{invoice_no}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Bill To: {{customer.name}}</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Date: {{invoice_date}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Item Code</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Unit Price</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Line Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>{{#each items}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>{{item_code}}</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>{{description}}</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>{{qty}}</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>{{unit_price}}</t>
-        </is>
-      </c>
-      <c r="E7" s="8">
-        <f>C7*D7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>{{/each}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Subtotal:</t>
-        </is>
-      </c>
-      <c r="E9" s="10">
-        <f>SUM(E7:E7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Scan to verify:</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>{{@qr 'https://verify.apex.corp/inv/' + invoice_no width=70 height=70}}</t>
-        </is>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="8" t="e">
+        <f>C8*D8</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D10" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="10" t="e">
+        <f>SUM(E8:E8)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1"/>
+    <hyperlink ref="B11" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: automatic string coercion in media tag expressions for numbers and strings
</commit_message>
<xml_diff>
--- a/templates/INVOICE_REPORT.xlsx
+++ b/templates/INVOICE_REPORT.xlsx
@@ -24,9 +24,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
-    <t>TAX INVOICE</t>
-  </si>
-  <si>
     <t>{{company.name}}</t>
   </si>
   <si>
@@ -75,16 +72,19 @@
     <t>Subtotal:</t>
   </si>
   <si>
-    <t>Scan to verify:</t>
-  </si>
-  <si>
     <t>{{#each invoices page_break=true}}</t>
   </si>
   <si>
-    <t>{{@barcode invoice_no format=code128 width=40 height=5}}</t>
-  </si>
-  <si>
-    <t>{{@qr 'https://verify.apex.corp/inv/' + invoice_no width=30 height=30}}</t>
+    <t>{{@qr 'https://verify.apex.corp/inv/' + invoice_no width=90 height=90}}</t>
+  </si>
+  <si>
+    <t>SALES TAX INVOICE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scan to verify: </t>
+  </si>
+  <si>
+    <t>{{@barcode invoice_no format=code128 width=150 height=40}}</t>
   </si>
 </sst>
 </file>
@@ -94,7 +94,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -132,6 +132,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1E293B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -182,7 +189,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -206,7 +213,15 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -510,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -522,67 +537,68 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>19</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="E2" s="11"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>1</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="E8" s="8" t="e">
         <f>C8*D8</f>
@@ -591,37 +607,40 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D10" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E10" s="10" t="e">
         <f>SUM(E8:E8)</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>15</v>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D2:E2"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1"/>
     <hyperlink ref="B11" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add text=true option to print human-readable text under barcode
</commit_message>
<xml_diff>
--- a/templates/INVOICE_REPORT.xlsx
+++ b/templates/INVOICE_REPORT.xlsx
@@ -84,7 +84,7 @@
     <t xml:space="preserve">Scan to verify: </t>
   </si>
   <si>
-    <t>{{@barcode invoice_no format=code128 width=150 height=40}}</t>
+    <t>{{@barcode 'helohelohelo' format=code128 width=150 height=40}}</t>
   </si>
 </sst>
 </file>
@@ -189,9 +189,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -216,11 +215,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -541,44 +549,47 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="B2" s="14"/>
+      <c r="D2" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="11"/>
+      <c r="E2" s="10"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="B3" s="11"/>
+      <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="B4" s="15"/>
+      <c r="D4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>8</v>
       </c>
     </row>
@@ -588,19 +599,19 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="8" t="e">
+      <c r="E8" s="7" t="e">
         <f>C8*D8</f>
         <v>#VALUE!</v>
       </c>
@@ -611,10 +622,10 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="10" t="e">
+      <c r="E10" s="9" t="e">
         <f>SUM(E8:E8)</f>
         <v>#VALUE!</v>
       </c>
@@ -633,8 +644,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1"/>

</xml_diff>

<commit_message>
docs: add modular enterprise documentation suite and update README
</commit_message>
<xml_diff>
--- a/templates/INVOICE_REPORT.xlsx
+++ b/templates/INVOICE_REPORT.xlsx
@@ -75,16 +75,16 @@
     <t>{{#each invoices page_break=true}}</t>
   </si>
   <si>
-    <t>{{@qr 'https://verify.apex.corp/inv/' + invoice_no width=90 height=90}}</t>
-  </si>
-  <si>
     <t>SALES TAX INVOICE</t>
   </si>
   <si>
     <t xml:space="preserve">Scan to verify: </t>
   </si>
   <si>
-    <t>{{@barcode 'helohelohelo' format=code128 width=150 height=40}}</t>
+    <t>{{@barcode 'helohelohelo' format=code128 width=180 height=50}}</t>
+  </si>
+  <si>
+    <t>~{{@qr 'https://verify.apex.corp/inv/' + invoice_no width=90 height=90}}</t>
   </si>
 </sst>
 </file>
@@ -218,9 +218,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -229,6 +226,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -549,12 +549,12 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="14"/>
+      <c r="A2" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="13"/>
       <c r="D2" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E2" s="10"/>
     </row>
@@ -568,10 +568,10 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="15"/>
+      <c r="B4" s="14"/>
       <c r="D4" s="2" t="s">
         <v>3</v>
       </c>
@@ -631,11 +631,11 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>17</v>
+      <c r="A11" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>